<commit_message>
Log prayer space submission from issue #1
</commit_message>
<xml_diff>
--- a/Prayer Space for Review.xlsx
+++ b/Prayer Space for Review.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,48 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-11T05:03:00Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>blueyeagle</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Test Mall</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Musollah</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Clear test submission from review workbook
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prayer Space for Review.xlsx
+++ b/Prayer Space for Review.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -480,48 +480,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-11T05:03:00Z</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>blueyeagle</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>#1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Test Mall</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Musollah</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log prayer space submission from issue #2
</commit_message>
<xml_diff>
--- a/Prayer Space for Review.xlsx
+++ b/Prayer Space for Review.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -480,6 +480,48 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-11T05:30:45Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>blueyeagle</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cintech 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Type: Prayer room</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Prayer room</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix submission parser: empty field no longer captures the next line
An empty 'Walk...:' value let \s* cross the newline and grab the Type line. Use [ \t]
around the colon so matches stay on one line. Corrected the stored Cintech 1 row.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prayer Space for Review.xlsx
+++ b/Prayer Space for Review.xlsx
@@ -506,11 +506,7 @@
           <t>Level 2</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Type: Prayer room</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Prayer room</t>

</xml_diff>